<commit_message>
Zerar a comissão do DEAN na folha de agosto
DEAN não recebe comissão sobre vendas. A rubrica passa a ser lançada
como zero em vez de puxar o valor apurado no InovaFarma, que fica apenas
como informação na aba BASE INOVAFARMA AGO.26.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
@@ -822,22 +822,18 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>DEAN: não recebe comissão sobre vendas — a rubrica fica zerada na folha. A comissão apurada no InovaFarma (R$ 975,65) aparece apenas na aba BASE, como informação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>PENDÊNCIAS — CONFIRMAR ANTES DE ENVIAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Horas extras e adicional noturno de agosto (apontamento do ponto).</t>
         </is>
       </c>
     </row>
@@ -849,7 +845,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Prêmio cota geral e prêmio pré-vencidos de agosto.</t>
+          <t>Horas extras e adicional noturno de agosto (apontamento do ponto).</t>
         </is>
       </c>
     </row>
@@ -861,7 +857,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Vales adiantados, convênio e faltas de agosto.</t>
+          <t>Prêmio cota geral e prêmio pré-vencidos de agosto.</t>
         </is>
       </c>
     </row>
@@ -873,7 +869,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>JOEL: informar o período de FÉRIAS de agosto/2026 para a contabilidade calcular férias, 1/3, média de comissões e o salário proporcional.</t>
+          <t>Vales adiantados, convênio e faltas de agosto.</t>
         </is>
       </c>
     </row>
@@ -885,7 +881,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>DEAN: apurou R$ 975,65 de comissão em agosto, mas não vinha recebendo comissão em folha — confirmar.</t>
+          <t>JOEL: informar o período de FÉRIAS de agosto/2026 para a contabilidade calcular férias, 1/3, média de comissões e o salário proporcional.</t>
         </is>
       </c>
     </row>
@@ -997,9 +993,9 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A1:B1"/>
@@ -1337,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1823,18 +1819,26 @@
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
+          <t>DEAN não recebe comissão em folha: no caso dele a comissão apurada acima é apenas informativa. Os incentivos continuam sendo lançados normalmente — confirmar se também ficam de fora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
           <t>JOEL: venda bruta de apenas R$ 5.057,69 porque esteve de FÉRIAS em agosto/2026 — a comissão apurada (R$ 103,31) corresponde só aos dias trabalhados.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:J12"/>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A23:J23"/>
     <mergeCell ref="A22:J22"/>
     <mergeCell ref="A21:J21"/>
     <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A24:J24"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2047,9 +2051,8 @@
           <t>COMISSÃO PRODUTOS (INOVAFARMA)</t>
         </is>
       </c>
-      <c r="B9" s="35">
-        <f>'BASE INOVAFARMA AGO.26'!F5</f>
-        <v/>
+      <c r="B9" s="35" t="n">
+        <v>0</v>
       </c>
       <c r="C9" s="35">
         <f>'BASE INOVAFARMA AGO.26'!F6</f>
@@ -2085,7 +2088,7 @@
       </c>
       <c r="K9" s="33" t="inlineStr">
         <is>
-          <t>Apurado no InovaFarma (aba BASE INOVAFARMA AGO.26). AGNOR: mantido o fixo de R$ 2.000,00 pela linha de complemento abaixo. DEAN: R$ 975,65 apurado — em jul/26 não houve lançamento de comissão para ele; confirmar.</t>
+          <t>Apurado no InovaFarma (aba BASE INOVAFARMA AGO.26). DEAN NÃO RECEBE COMISSÃO — lançado zero (o apurado dele fica só como informação na aba BASE). AGNOR: mantido o fixo de R$ 2.000,00 pela linha de complemento abaixo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adicionar demonstrativo individual e tratar as férias do JOEL
- Nova aba GANHOS DO COLABORADOR: lista suspensa com os nomes e o
  demonstrativo da pessoa escolhida, montado por INDEX/MATCH sobre a aba
  HOLERITE AGO.26, mais o resumo de vendas do InovaFarma; configurada
  para imprimir em uma página
- JOEL: férias de 01 a 31/08/2026 já pagas no início de agosto — salário
  e desconto de vale-transporte zerados, rubricas de férias mantidas
  apenas como referência e alerta sobre a comissão apurada no código dele
- DEAN mantém os incentivos; observações ajustadas

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
@@ -13,12 +13,14 @@
     <sheet name="HOLERITE AGO.26" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="JULHO.26 REVISADO" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="LISTA CONTABILIDADE" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="GANHOS DO COLABORADOR" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BASE INOVAFARMA AGO.26'!$A$4:$J$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'HOLERITE AGO.26'!$A$4:$K$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'JULHO.26 REVISADO'!$A$4:$K$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'LISTA CONTABILIDADE'!$A$4:$E$187</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'GANHOS DO COLABORADOR'!$A$1:$D$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +32,7 @@
     <numFmt numFmtId="164" formatCode="R$ #,##0.00;-R$ #,##0.00;&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,6 +117,24 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
@@ -193,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -202,7 +222,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -276,6 +296,13 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -641,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -810,7 +837,7 @@
       <c r="A23" s="4" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>JOEL: esteve de férias em agosto/2026 — por isso a venda e a comissão do mês ficaram baixas.</t>
+          <t>JOEL: férias de 01 a 31/08/2026 (mês inteiro), já pagas em recibo próprio no início de agosto. Neste holerite ele fica sem salário e sem desconto de vale-transporte; férias e 1/3 NÃO se repetem aqui.</t>
         </is>
       </c>
     </row>
@@ -826,7 +853,7 @@
       <c r="A25" s="4" t="inlineStr"/>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>DEAN: não recebe comissão sobre vendas — a rubrica fica zerada na folha. A comissão apurada no InovaFarma (R$ 975,65) aparece apenas na aba BASE, como informação.</t>
+          <t>DEAN: não recebe comissão sobre vendas — a rubrica fica zerada na folha (a apurada, R$ 975,65, aparece só na aba BASE). Os incentivos dele continuam sendo pagos normalmente.</t>
         </is>
       </c>
     </row>
@@ -881,7 +908,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>JOEL: informar o período de FÉRIAS de agosto/2026 para a contabilidade calcular férias, 1/3, média de comissões e o salário proporcional.</t>
+          <t>JOEL: o código dele registrou R$ 103,31 de comissão mesmo com o mês inteiro de férias — conferir quem operou o código e zerar a rubrica se as vendas não forem dele.</t>
         </is>
       </c>
     </row>
@@ -893,7 +920,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Comissões de PDV antigos, que em julho eram somadas à comissão do sistema.</t>
+          <t>JOEL: confirmar se sobra algum desconto para agosto (convênio, vale ou adiantamento) ou se o holerite dele fica zerado.</t>
         </is>
       </c>
     </row>
@@ -905,7 +932,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Desconto de vale-transporte: vem sendo lançado R$ 84,29; 6% do salário de R$ 1.621,00 seria R$ 97,26.</t>
+          <t>Comissões de PDV antigos, que em julho eram somadas à comissão do sistema.</t>
         </is>
       </c>
     </row>
@@ -917,37 +944,41 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
+          <t>Desconto de vale-transporte: vem sendo lançado R$ 84,29; 6% do salário de R$ 1.621,00 seria R$ 97,26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
           <t>DSR de julho/2026 foi calculado com o fator de agosto (5/26) em vez de 4/27 — ver aba JULHO.26 REVISADO e decidir se ajusta em setembro.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO TÉCNICA</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="4" t="inlineStr"/>
-      <c r="B35" s="5" t="inlineStr">
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>As células de total e de cálculo são fórmulas. Ao abrir o arquivo no Excel ou no Google Planilhas os valores aparecem calculados automaticamente; em visualizadores simples (prévia de celular, por exemplo) elas podem aparecer em branco até o arquivo ser aberto de fato.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>ABAS DO ARQUIVO</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="17" customHeight="1">
-      <c r="A37" s="4" t="inlineStr"/>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -955,7 +986,7 @@
       <c r="A38" s="4" t="inlineStr"/>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista por funcionário.</t>
+          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -963,7 +994,7 @@
       <c r="A39" s="4" t="inlineStr"/>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
+          <t>GANHOS DO COLABORADOR — escolha o nome na lista e saia o demonstrativo individual, pronto para imprimir/mandar.</t>
         </is>
       </c>
     </row>
@@ -971,7 +1002,7 @@
       <c r="A40" s="4" t="inlineStr"/>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>JULHO.26 REVISADO — a folha de julho reorganizada e conferida (valores pagos preservados).</t>
+          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista por funcionário.</t>
         </is>
       </c>
     </row>
@@ -979,12 +1010,28 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
+          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>JULHO.26 REVISADO — a folha de julho reorganizada e conferida (valores pagos preservados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="17" customHeight="1">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
           <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="7" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Documento gerado a partir da planilha CONISSÕES PLAN.AGOSTO/JULHO ARRAIAL 2026 e do relatório de comissões do InovaFarma.</t>
         </is>
@@ -997,10 +1044,10 @@
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1819,14 +1866,14 @@
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>DEAN não recebe comissão em folha: no caso dele a comissão apurada acima é apenas informativa. Os incentivos continuam sendo lançados normalmente — confirmar se também ficam de fora.</t>
+          <t>DEAN não recebe comissão em folha: no caso dele a comissão apurada acima é apenas informativa. Os incentivos dele continuam sendo lançados normalmente.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>JOEL: venda bruta de apenas R$ 5.057,69 porque esteve de FÉRIAS em agosto/2026 — a comissão apurada (R$ 103,31) corresponde só aos dias trabalhados.</t>
+          <t>JOEL: esteve de FÉRIAS de 01 a 31/08/2026 (mês inteiro), mas o código dele registrou R$ 5.057,69 de venda bruta e R$ 103,31 de comissão — conferir quem operou o código no período.</t>
         </is>
       </c>
     </row>
@@ -1971,7 +2018,7 @@
         <v>1621</v>
       </c>
       <c r="E6" s="31" t="n">
-        <v>1621</v>
+        <v>0</v>
       </c>
       <c r="F6" s="31" t="n">
         <v>1621</v>
@@ -1991,7 +2038,7 @@
       </c>
       <c r="K6" s="33" t="inlineStr">
         <is>
-          <t>Piso 2026 R$ 1.621,00. CAMILA: admitida em jul/26 (salário proporcional naquele mês); agosto é o 1º mês completo. JOEL: ajustar aos dias trabalhados por conta das férias.</t>
+          <t>Piso 2026 R$ 1.621,00. CAMILA: admitida em jul/26 (salário proporcional naquele mês); agosto é o 1º mês completo. JOEL: zerado — esteve de férias de 01 a 31/08/2026, sem dias trabalhados no mês.</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2135,7 @@
       </c>
       <c r="K9" s="33" t="inlineStr">
         <is>
-          <t>Apurado no InovaFarma (aba BASE INOVAFARMA AGO.26). DEAN NÃO RECEBE COMISSÃO — lançado zero (o apurado dele fica só como informação na aba BASE). AGNOR: mantido o fixo de R$ 2.000,00 pela linha de complemento abaixo.</t>
+          <t>Apurado no InovaFarma (aba BASE INOVAFARMA AGO.26). JOEL: R$ 103,31 apurados no código dele mesmo estando de férias o mês inteiro — conferir quem fez essas vendas e zerar se não forem dele. DEAN NÃO RECEBE COMISSÃO — lançado zero (o apurado dele fica só como informação na aba BASE). AGNOR: mantido o fixo de R$ 2.000,00 pela linha de complemento abaixo.</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2384,7 @@
       </c>
       <c r="K17" s="33" t="inlineStr">
         <is>
-          <t>JOEL esteve de FÉRIAS em agosto/2026 — informar o período para a contabilidade calcular férias, média de comissões e o salário proporcional aos dias trabalhados.</t>
+          <t>JOEL: férias de 01 a 31/08/2026, JÁ PAGAS em recibo próprio no início de agosto — NÃO lançar de novo neste holerite. Linha mantida só para o caso de outras férias.</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2408,7 @@
       </c>
       <c r="K18" s="33" t="inlineStr">
         <is>
-          <t>Calculado pela contabilidade sobre o valor das férias.</t>
+          <t>JOEL: também já pago com as férias no início de agosto. Linha mantida para eventuais férias de outros meses.</t>
         </is>
       </c>
     </row>
@@ -2705,9 +2752,7 @@
       <c r="D28" s="31" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="E28" s="31" t="n">
-        <v>-84.29000000000001</v>
-      </c>
+      <c r="E28" s="31" t="n"/>
       <c r="F28" s="31" t="n">
         <v>-84.29000000000001</v>
       </c>
@@ -2722,7 +2767,7 @@
       </c>
       <c r="K28" s="33" t="inlineStr">
         <is>
-          <t>Valor praticado em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada.</t>
+          <t>Valor praticado em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada. JOEL: zerado, mês inteiro de férias.</t>
         </is>
       </c>
     </row>
@@ -8134,4 +8179,446 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DEMONSTRATIVO DE GANHOS DO COLABORADOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Competência AGOSTO/2026 · Pagamento em 05/09/2026 · Farmácia Tropical Multi Econômica</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Escolha o colaborador:</t>
+        </is>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>DEAN</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Troque o nome aqui e a tabela abaixo muda sozinha — é o relatório para mandar para cada um.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>PROVENTOS</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="29" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Salário base</t>
+        </is>
+      </c>
+      <c r="C7" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$I$6,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Adicional noturno</t>
+        </is>
+      </c>
+      <c r="C8" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$7:$I$7,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Horas extras</t>
+        </is>
+      </c>
+      <c r="C9" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$8:$I$8,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Comissão sobre vendas</t>
+        </is>
+      </c>
+      <c r="C10" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$11:$I$11,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Repouso remunerado / DSR</t>
+        </is>
+      </c>
+      <c r="C11" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$12:$I$12,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Auxílio gerência</t>
+        </is>
+      </c>
+      <c r="C12" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$13:$I$13,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Adicional prêmio meta caixa</t>
+        </is>
+      </c>
+      <c r="C13" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$14:$I$14,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Prêmio cota geral</t>
+        </is>
+      </c>
+      <c r="C14" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$15:$I$15,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Prêmio pré-vencidos</t>
+        </is>
+      </c>
+      <c r="C15" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$16:$I$16,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Férias</t>
+        </is>
+      </c>
+      <c r="C16" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$17:$I$17,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>1/3 constitucional de férias</t>
+        </is>
+      </c>
+      <c r="C17" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$18:$I$18,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Incentivo aplicações</t>
+        </is>
+      </c>
+      <c r="C18" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$19:$I$19,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Incentivo vitaminas</t>
+        </is>
+      </c>
+      <c r="C19" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$20:$I$20,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Outros incentivos</t>
+        </is>
+      </c>
+      <c r="C20" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$21:$I$21,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL DE PROVENTOS</t>
+        </is>
+      </c>
+      <c r="C21" s="43">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$22:$I$22,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="19" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>DESCONTOS</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="n"/>
+      <c r="D22" s="29" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Adiantamento / vales</t>
+        </is>
+      </c>
+      <c r="C23" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$24:$I$24,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Adiantamento de incentivos e aplicações</t>
+        </is>
+      </c>
+      <c r="C24" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$25:$I$25,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Convênio</t>
+        </is>
+      </c>
+      <c r="C25" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$26:$I$26,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="30" t="inlineStr">
+        <is>
+          <t>Faltas / atrasos</t>
+        </is>
+      </c>
+      <c r="C26" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$27:$I$27,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Vale transporte 6%</t>
+        </is>
+      </c>
+      <c r="C27" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$28:$I$28,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>INSS</t>
+        </is>
+      </c>
+      <c r="C28" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$29:$I$29,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>IRRF</t>
+        </is>
+      </c>
+      <c r="C29" s="35">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$30:$I$30,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL DE DESCONTOS</t>
+        </is>
+      </c>
+      <c r="C30" s="43">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$31:$I$31,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>LÍQUIDO</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="29" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="50" t="inlineStr">
+        <is>
+          <t>LÍQUIDO A RECEBER EM 05/09/2026</t>
+        </is>
+      </c>
+      <c r="C32" s="51">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$33:$I$33,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$I$4,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="52" t="inlineStr">
+        <is>
+          <t>Vendas do colaborador no mês (InovaFarma):</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>Venda bruta</t>
+        </is>
+      </c>
+      <c r="C35" s="35">
+        <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$C$5:$C$12,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$12,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>Descontos concedidos</t>
+        </is>
+      </c>
+      <c r="C36" s="35">
+        <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$D$5:$D$12,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$12,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>Venda líquida</t>
+        </is>
+      </c>
+      <c r="C37" s="35">
+        <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$E$5:$E$12,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$12,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>Comissão apurada</t>
+        </is>
+      </c>
+      <c r="C38" s="35">
+        <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$F$5:$F$12,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$12,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>Total de incentivos</t>
+        </is>
+      </c>
+      <c r="C39" s="35">
+        <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$J$5:$J$12,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$12,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>A comissão apurada acima é a apuração do sistema. O que entra na folha é a linha "Comissão sobre vendas" — pode ser diferente (valor fixo acordado, PDV antigos ou quem não recebe comissão).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Os valores de INSS e IRRF são calculados pela contabilidade e só aparecem aqui depois de preenchidos na aba HOLERITE AGO.26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Para mandar para o colaborador: selecione o nome acima e imprima esta aba em PDF (ou tire um print).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Na aba LISTA CONTABILIDADE também dá para filtrar por FUNCIONÁRIO e ver só os lançamentos de uma pessoa.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Escolha um nome da lista." promptTitle="Colaborador" prompt="Selecione o colaborador para ver os ganhos dele." type="list">
+      <formula1>"DEAN,AGNOR,EDEY,JOEL,VALÉRIA,SARA,CAMILA,NATI"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Explicar a comissão do JOEL pelo acordo interno de férias
Pelo acordo interno ele saiu em 04/08 e volta em 04/09, embora o recibo
de férias tenha saído como 01 a 31/08. A comissão de R$ 103,31 vem das
vendas dos dias 01 e 02/08 e deixa de ser tratada como divergência.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
@@ -837,7 +837,7 @@
       <c r="A23" s="4" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>JOEL: férias de 01 a 31/08/2026 (mês inteiro), já pagas em recibo próprio no início de agosto. Neste holerite ele fica sem salário e sem desconto de vale-transporte; férias e 1/3 NÃO se repetem aqui.</t>
+          <t>JOEL: por acordo interno saiu em 04/08 e volta em 04/09, mas o recibo de férias saiu como 01 a 31/08 e já foi pago no início de agosto. Por isso ele tem comissão dos dias 01 e 02/08 (R$ 103,31) e fica sem salário e sem desconto de vale-transporte neste holerite; férias e 1/3 NÃO se repetem aqui.</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>JOEL: o código dele registrou R$ 103,31 de comissão mesmo com o mês inteiro de férias — conferir quem operou o código e zerar a rubrica se as vendas não forem dele.</t>
+          <t>JOEL: confirmar se há algum desconto para agosto (convênio, vale ou adiantamento) — hoje o holerite dele fica só com a comissão de R$ 103,31 e o DSR.</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>JOEL: confirmar se sobra algum desconto para agosto (convênio, vale ou adiantamento) ou se o holerite dele fica zerado.</t>
+          <t>JOEL: como o retorno é em 04/09, o vale-transporte de setembro deve ser proporcional e o holerite de setembro ainda pega os dias 01 a 03/09 de férias, já pagos no recibo de agosto.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>JOEL: esteve de FÉRIAS de 01 a 31/08/2026 (mês inteiro), mas o código dele registrou R$ 5.057,69 de venda bruta e R$ 103,31 de comissão — conferir quem operou o código no período.</t>
+          <t>JOEL: vendeu R$ 3.684,97 nos dias 01 e 02/08 e saiu de férias em 04/08 (retorno em 04/09) — daí a comissão de R$ 103,31. Constam ainda 2 itens de R$ 11,68 em 07/08 no código dele.</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="K6" s="33" t="inlineStr">
         <is>
-          <t>Piso 2026 R$ 1.621,00. CAMILA: admitida em jul/26 (salário proporcional naquele mês); agosto é o 1º mês completo. JOEL: zerado — esteve de férias de 01 a 31/08/2026, sem dias trabalhados no mês.</t>
+          <t>Piso 2026 R$ 1.621,00. CAMILA: admitida em jul/26 (salário proporcional naquele mês); agosto é o 1º mês completo. JOEL: zerado — trabalhou de 01 a 03/08 mas esses dias já estão dentro do recibo de férias (01 a 31/08); se a empresa decidir pagá-los à parte, lançar aqui.</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="K9" s="33" t="inlineStr">
         <is>
-          <t>Apurado no InovaFarma (aba BASE INOVAFARMA AGO.26). JOEL: R$ 103,31 apurados no código dele mesmo estando de férias o mês inteiro — conferir quem fez essas vendas e zerar se não forem dele. DEAN NÃO RECEBE COMISSÃO — lançado zero (o apurado dele fica só como informação na aba BASE). AGNOR: mantido o fixo de R$ 2.000,00 pela linha de complemento abaixo.</t>
+          <t>Apurado no InovaFarma (aba BASE INOVAFARMA AGO.26). JOEL: R$ 103,31 das vendas dele nos dias 01 e 02/08, antes de sair de férias em 04/08 (o recibo de férias saiu como 01 a 31/08). DEAN NÃO RECEBE COMISSÃO — lançado zero (o apurado dele fica só como informação na aba BASE). AGNOR: mantido o fixo de R$ 2.000,00 pela linha de complemento abaixo.</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="K17" s="33" t="inlineStr">
         <is>
-          <t>JOEL: férias de 01 a 31/08/2026, JÁ PAGAS em recibo próprio no início de agosto — NÃO lançar de novo neste holerite. Linha mantida só para o caso de outras férias.</t>
+          <t>JOEL: recibo de férias de 01 a 31/08/2026, JÁ PAGO no início de agosto — NÃO lançar de novo aqui. Pelo acordo interno ele saiu em 04/08 e volta em 04/09.</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="K28" s="33" t="inlineStr">
         <is>
-          <t>Valor praticado em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada. JOEL: zerado, mês inteiro de férias.</t>
+          <t>Valor praticado em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada. JOEL: zerado, mês de férias.</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="K35" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER com as passagens compradas para setembro/2026.</t>
+          <t>PREENCHER com as passagens compradas para setembro/2026. JOEL: só a partir de 04/09, quando volta das férias.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lançar as horas das madrugadas de VALÉRIA e AGNOR
Cada madrugada foi jornada normal de 8 horas com intervalo: VALÉRIA com
2 madrugadas (16 h) e AGNOR com 3 (24 h), lançadas como horas noturnas
na aba PONTO AGO.26.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_pgto_05-09-2026.xlsx
@@ -857,7 +857,7 @@
       <c r="A25" s="4" t="inlineStr"/>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>VALÉRIA: 2 madrugadas com folga no dia seguinte — cabe só o adicional noturno; falta informar as horas.</t>
+          <t>VALÉRIA: 2 madrugadas de 8 horas (16 h) com folga no dia seguinte → R$ 23,58 de adicional noturno.</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       <c r="A26" s="4" t="inlineStr"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>AGNOR: 3 madrugadas com folga — cabe só o adicional noturno; falta informar as horas.</t>
+          <t>AGNOR: 3 madrugadas de 8 horas (24 h) com folga → R$ 35,37 de adicional noturno.</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>VALÉRIA e AGNOR: informar na aba PONTO AGO.26 quantas horas noturnas tiveram as madrugadas trabalhadas (2 e 3 madrugadas).</t>
+          <t>VALÉRIA e AGNOR: as madrugadas entraram como 8 horas cada (jornada normal com intervalo). Se só parte dessas horas ficou entre 22h e 5h, ajustar a quantidade na aba PONTO AGO.26.</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Conforme jul/2026 — conferir apontamento do ponto.</t>
+          <t>Referência de jul/2026. O valor efetivo é lançado na aba PONTO AGO.26 — conferir com o apontamento.</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
         <v/>
       </c>
       <c r="K12" s="33">
-        <f> (comissão total + horas extras) × 5 domingos ÷ 26 dias úteis de agosto/2026 (fator na aba PARÂMETROS).</f>
+        <f> (comissão total + horas extras) × 5 domingos ÷ 26 dias úteis de agosto/2026 (fator na aba PARÂMETROS). A linha HORAS EXTRAS inclui o feriado trabalhado vindo da aba PONTO AGO.26.</f>
         <v/>
       </c>
     </row>
@@ -9224,7 +9224,9 @@
           <t>Adicional noturno</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
+      <c r="C12" s="9" t="n">
+        <v>16</v>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>horas</t>
@@ -9249,7 +9251,7 @@
       </c>
       <c r="I12" s="33" t="inlineStr">
         <is>
-          <t>2 madrugadas trabalhadas, com folga normal no dia seguinte — cabe só o adicional noturno. INFORMAR o total de horas noturnas das 2 madrugadas.</t>
+          <t>2 madrugadas de jornada normal de 8 horas com intervalo (2 × 8 = 16 h), com folga normal no dia seguinte — cabe só o adicional noturno.</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9266,9 @@
           <t>Adicional noturno</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
+      <c r="C13" s="9" t="n">
+        <v>24</v>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>horas</t>
@@ -9289,7 +9293,7 @@
       </c>
       <c r="I13" s="33" t="inlineStr">
         <is>
-          <t>3 madrugadas trabalhadas, com folga normal — cabe só o adicional noturno. INFORMAR o total de horas noturnas das 3 madrugadas.</t>
+          <t>3 madrugadas de jornada normal de 8 horas com intervalo (3 × 8 = 24 h), com folga normal — cabe só o adicional noturno.</t>
         </is>
       </c>
     </row>

</xml_diff>